<commit_message>
nesw line in excel
</commit_message>
<xml_diff>
--- a/80_uts_test.xlsx
+++ b/80_uts_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://resoca-my.sharepoint.com/personal/martin_troup_grandest_chambagri_fr/Documents/VADEMECUM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E60FDC74-524D-4324-AF8B-8408B1DC2403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{E60FDC74-524D-4324-AF8B-8408B1DC2403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D68D3C45-B971-4E33-9D29-956D7CB5E4C6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6EDEA7E0-CF20-495E-8FE7-C7395E990510}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16484" uniqueCount="16424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16506" uniqueCount="16439">
   <si>
     <t>no_uts</t>
   </si>
@@ -49311,6 +49311,51 @@
   </si>
   <si>
     <t>nvoProfil_UTS_9412.jpg</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>rendisols</t>
+  </si>
+  <si>
+    <t>Sol forestier superficiel argileux sur calcaires oxfordiens</t>
+  </si>
+  <si>
+    <t>RENDISOL ARGILEUX FORESTIER</t>
+  </si>
+  <si>
+    <t>Aci</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>CALCAIRES DURS SUBRECIFAUX ET CALC. ARG. EN BANCS</t>
+  </si>
+  <si>
+    <t>C:\Users\pouzencs44r\Desktop\Carto_VADEMECUM\script_Vademecum\choix_uts \GER_carte_uts\2014.jpeg</t>
+  </si>
+  <si>
+    <t>2014.jpeg</t>
+  </si>
+  <si>
+    <t>C:\Users\pouzencs44r\Desktop\Carto_VADEMECUM\script_Vademecum\roues des services\roue_agro_UTS_2014.jpg</t>
+  </si>
+  <si>
+    <t>roue_agro_UTS_2014.jpg</t>
+  </si>
+  <si>
+    <t>C:\Users\pouzencs44r\Desktop\Carto_VADEMECUM\script_Vademecum\roues des services\roue_service_UTS_2014.jpg</t>
+  </si>
+  <si>
+    <t>roue_service_UTS_2014.jpg</t>
+  </si>
+  <si>
+    <t>C:/Users/pouzencs44r/Desktop/Carto_VADEMECUM/script_Vademecum/profils de sols/\nvoProfil_UTS_2014.jpg</t>
+  </si>
+  <si>
+    <t>nvoProfil_UTS_2014.jpg</t>
   </si>
 </sst>
 </file>
@@ -49682,7 +49727,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A480FD3-E604-4FCD-A1B0-A718D691056D}">
-  <dimension ref="A1:XFD3"/>
+  <dimension ref="A1:XFD4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:16384" x14ac:dyDescent="0.3">
@@ -99470,6 +99515,113 @@
         <v>16423</v>
       </c>
     </row>
+    <row r="4" spans="1:16384" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16424</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>16425</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16388</v>
+      </c>
+      <c r="J4" t="s">
+        <v>16426</v>
+      </c>
+      <c r="K4" t="s">
+        <v>16427</v>
+      </c>
+      <c r="L4" t="s">
+        <v>16388</v>
+      </c>
+      <c r="M4" t="s">
+        <v>16428</v>
+      </c>
+      <c r="N4" t="s">
+        <v>16429</v>
+      </c>
+      <c r="S4" t="s">
+        <v>16388</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>16430</v>
+      </c>
+      <c r="AJ4">
+        <v>0</v>
+      </c>
+      <c r="AP4">
+        <v>490</v>
+      </c>
+      <c r="AV4">
+        <v>0</v>
+      </c>
+      <c r="BA4">
+        <v>0</v>
+      </c>
+      <c r="BF4">
+        <v>0</v>
+      </c>
+      <c r="BK4">
+        <v>6.2</v>
+      </c>
+      <c r="BQ4">
+        <v>30</v>
+      </c>
+      <c r="BW4">
+        <v>65</v>
+      </c>
+      <c r="CH4">
+        <v>0</v>
+      </c>
+      <c r="CX4">
+        <v>20</v>
+      </c>
+      <c r="EA4" t="s">
+        <v>16428</v>
+      </c>
+      <c r="EG4" t="s">
+        <v>16427</v>
+      </c>
+      <c r="EM4" t="s">
+        <v>16397</v>
+      </c>
+      <c r="ES4">
+        <v>222579</v>
+      </c>
+      <c r="EY4">
+        <v>39891.717127999997</v>
+      </c>
+      <c r="FQ4" t="s">
+        <v>16399</v>
+      </c>
+      <c r="FW4" t="s">
+        <v>16431</v>
+      </c>
+      <c r="FX4" t="s">
+        <v>16432</v>
+      </c>
+      <c r="FY4" t="s">
+        <v>16433</v>
+      </c>
+      <c r="FZ4" t="s">
+        <v>16434</v>
+      </c>
+      <c r="GA4" t="s">
+        <v>16435</v>
+      </c>
+      <c r="GB4" t="s">
+        <v>16436</v>
+      </c>
+      <c r="GH4" t="s">
+        <v>16437</v>
+      </c>
+      <c r="GM4" t="s">
+        <v>16438</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>